<commit_message>
Regenerate templates, Sentinel workbook text and OG images as ScopeSense
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/rfp-evaluation-criteria-worksheet.xlsx
+++ b/apps/web/public/templates/rfp-evaluation-criteria-worksheet.xlsx
@@ -446,7 +446,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RFP evaluation criteria worksheet (ScopeWise)</t>
+          <t>RFP evaluation criteria worksheet (ScopeSense)</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>This worksheet is guidance, not legal advice. https://scopewise.assessiq.in/use-cases/rfp-review</t>
+          <t>This worksheet is guidance, not legal advice. https://scopesense.in/use-cases/rfp-review</t>
         </is>
       </c>
     </row>

</xml_diff>